<commit_message>
v3.6.8: GT tuning, RL env
</commit_message>
<xml_diff>
--- a/results/SamChigome/analysis/n_10/AllData.xlsx
+++ b/results/SamChigome/analysis/n_10/AllData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\owuor\owProjects\StructuralGT\results\SamChigome\analysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\owuor\owProjects\StructuralGT\results\SamChigome\analysis\n_10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8B9FEAD-44E5-401B-A4B4-A7F40F0ABCAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD345C3C-8067-4842-921F-AD6DC480F469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="8" activeTab="14" xr2:uid="{E8351862-8131-4AC1-82A9-213539580791}"/>
+    <workbookView xWindow="360" yWindow="375" windowWidth="27690" windowHeight="10455" firstSheet="9" activeTab="14" xr2:uid="{E8351862-8131-4AC1-82A9-213539580791}"/>
   </bookViews>
   <sheets>
     <sheet name="SGT Descriptors" sheetId="2" r:id="rId1"/>
@@ -4887,8 +4887,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{B89027AB-5D9D-4421-B80B-99DB9E634340}" name="Table6" displayName="Table6" ref="A5:B9" totalsRowShown="0">
-  <autoFilter ref="A5:B9" xr:uid="{B89027AB-5D9D-4421-B80B-99DB9E634340}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{B89027AB-5D9D-4421-B80B-99DB9E634340}" name="Table6" displayName="Table6" ref="A2:B6" totalsRowShown="0">
+  <autoFilter ref="A2:B6" xr:uid="{B89027AB-5D9D-4421-B80B-99DB9E634340}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{70364C0B-1320-4A7E-AD30-25F8414086FE}" name="a"/>
     <tableColumn id="2" xr3:uid="{AEDFE533-B065-41FB-A636-6D5C56171853}" name="k"/>
@@ -6402,46 +6402,46 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D20DC337-6F2B-4C6F-A1A5-B5E5DC0F7BCC}">
-  <dimension ref="A5:B9"/>
+  <dimension ref="A2:B6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2.77</v>
+      </c>
+      <c r="B3">
+        <v>0.97</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2.41</v>
+      </c>
+      <c r="B4">
+        <v>0.95</v>
+      </c>
+    </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>34</v>
-      </c>
-      <c r="B5" t="s">
-        <v>35</v>
+      <c r="A5">
+        <v>2.76</v>
+      </c>
+      <c r="B5">
+        <v>0.96</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>2.77</v>
+        <v>2.75</v>
       </c>
       <c r="B6">
-        <v>0.97</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>2.41</v>
-      </c>
-      <c r="B7">
-        <v>0.95</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>2.76</v>
-      </c>
-      <c r="B8">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>2.75</v>
-      </c>
-      <c r="B9">
         <v>0.95</v>
       </c>
     </row>

</xml_diff>